<commit_message>
Feat: Migração inicial para banco de dados adicionando as funcionalidades de Comrpas, Vendas, CLientes e participantes, atualização do README
</commit_message>
<xml_diff>
--- a/dados/Controle.xlsx
+++ b/dados/Controle.xlsx
@@ -1154,7 +1154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4629,6 +4629,786 @@
         <v>46047.54166666666</v>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B134" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C134" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D134" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="E134" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F134" s="9" t="n">
+        <v>45682.54166666666</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="inlineStr">
+        <is>
+          <t>Compra A</t>
+        </is>
+      </c>
+      <c r="B135" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C135" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D135" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E135" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F135" s="9" t="n">
+        <v>46047.375</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="inlineStr">
+        <is>
+          <t>Compra B</t>
+        </is>
+      </c>
+      <c r="B136" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C136" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D136" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E136" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F136" s="9" t="n">
+        <v>46047.41666666666</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B137" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C137" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D137" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E137" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F137" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B138" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C138" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D138" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E138" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F138" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="inlineStr">
+        <is>
+          <t>Compra C</t>
+        </is>
+      </c>
+      <c r="B139" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C139" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D139" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E139" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F139" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B140" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C140" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D140" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="E140" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F140" s="9" t="n">
+        <v>45682.54166666666</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t>Compra A</t>
+        </is>
+      </c>
+      <c r="B141" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C141" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D141" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E141" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F141" s="9" t="n">
+        <v>46047.375</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="inlineStr">
+        <is>
+          <t>Compra B</t>
+        </is>
+      </c>
+      <c r="B142" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C142" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D142" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E142" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F142" s="9" t="n">
+        <v>46047.41666666666</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B143" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C143" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D143" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E143" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F143" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B144" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C144" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D144" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E144" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F144" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="inlineStr">
+        <is>
+          <t>Compra C</t>
+        </is>
+      </c>
+      <c r="B145" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C145" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D145" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E145" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F145" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B146" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C146" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D146" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="E146" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F146" s="9" t="n">
+        <v>45682.54166666666</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t>Compra A</t>
+        </is>
+      </c>
+      <c r="B147" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C147" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D147" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E147" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F147" s="9" t="n">
+        <v>46047.375</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="inlineStr">
+        <is>
+          <t>Compra B</t>
+        </is>
+      </c>
+      <c r="B148" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C148" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D148" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E148" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F148" s="9" t="n">
+        <v>46047.41666666666</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B149" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C149" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D149" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E149" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F149" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B150" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C150" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D150" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E150" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F150" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="inlineStr">
+        <is>
+          <t>Compra C</t>
+        </is>
+      </c>
+      <c r="B151" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C151" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D151" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E151" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F151" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B152" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C152" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D152" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="E152" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F152" s="9" t="n">
+        <v>45682.54166666666</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="inlineStr">
+        <is>
+          <t>Compra A</t>
+        </is>
+      </c>
+      <c r="B153" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C153" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D153" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E153" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F153" s="9" t="n">
+        <v>46047.375</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="inlineStr">
+        <is>
+          <t>Compra B</t>
+        </is>
+      </c>
+      <c r="B154" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C154" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D154" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E154" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F154" s="9" t="n">
+        <v>46047.41666666666</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B155" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C155" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D155" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E155" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F155" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B156" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C156" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D156" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E156" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F156" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="inlineStr">
+        <is>
+          <t>Compra C</t>
+        </is>
+      </c>
+      <c r="B157" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C157" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D157" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F157" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B158" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C158" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D158" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="E158" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F158" s="9" t="n">
+        <v>45682.54166666666</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>Compra A</t>
+        </is>
+      </c>
+      <c r="B159" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C159" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D159" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E159" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F159" s="9" t="n">
+        <v>46047.375</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t>Compra B</t>
+        </is>
+      </c>
+      <c r="B160" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C160" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D160" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E160" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F160" s="9" t="n">
+        <v>46047.41666666666</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B161" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C161" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D161" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E161" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F161" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="B162" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C162" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D162" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E162" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F162" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="inlineStr">
+        <is>
+          <t>Compra C</t>
+        </is>
+      </c>
+      <c r="B163" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C163" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D163" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E163" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F163" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4640,7 +5420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7849,6 +8629,655 @@
         <v>31</v>
       </c>
       <c r="G104" s="9" t="n">
+        <v>46047.58333333334</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B105" s="1" t="inlineStr">
+        <is>
+          <t>Venda A</t>
+        </is>
+      </c>
+      <c r="C105" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="D105" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E105" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F105" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G105" s="9" t="n">
+        <v>46047.45833333334</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>Jose</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C106" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D106" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E106" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F106" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G106" s="9" t="n">
+        <v>46047.5</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C107" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D107" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E107" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F107" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G107" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C108" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D108" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E108" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G108" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C109" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D109" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E109" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G109" s="9" t="n">
+        <v>46047.58333333334</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>Jose</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C110" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D110" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E110" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G110" s="9" t="n">
+        <v>46047.5</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B111" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C111" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D111" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E111" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G111" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B112" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C112" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D112" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E112" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G112" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B113" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C113" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D113" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E113" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G113" s="9" t="n">
+        <v>46047.58333333334</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>Jose</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C114" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D114" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E114" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G114" s="9" t="n">
+        <v>46047.5</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B115" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C115" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D115" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E115" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G115" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B116" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C116" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D116" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E116" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G116" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B117" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C117" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D117" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E117" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G117" s="9" t="n">
+        <v>46047.58333333334</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="inlineStr">
+        <is>
+          <t>Jose</t>
+        </is>
+      </c>
+      <c r="B118" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C118" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D118" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E118" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G118" s="9" t="n">
+        <v>46047.5</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B119" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C119" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D119" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E119" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F119" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G119" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B120" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C120" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E120" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F120" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G120" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E121" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F121" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G121" s="9" t="n">
+        <v>46047.58333333334</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="inlineStr">
+        <is>
+          <t>Jose</t>
+        </is>
+      </c>
+      <c r="B122" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C122" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D122" s="1" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E122" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F122" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G122" s="9" t="n">
+        <v>46047.5</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B123" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C123" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D123" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E123" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F123" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G123" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B124" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C124" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D124" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E124" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F124" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G124" s="9" t="n">
+        <v>46047.54166666666</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E125" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F125" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G125" s="9" t="n">
         <v>46047.58333333334</v>
       </c>
     </row>
@@ -7906,7 +9335,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>12558</v>
+        <v>13048</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>31</v>
@@ -7924,7 +9353,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>30</v>
@@ -7942,7 +9371,7 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>31</v>
@@ -7960,7 +9389,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>31</v>
@@ -7976,7 +9405,7 @@
         <v>36</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>31</v>
@@ -7993,7 +9422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10418,6 +11847,546 @@
         <v>46167.54166666666</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B90" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C90" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E90" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F90" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G90" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B91" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C91" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E91" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F91" s="8" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G91" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B92" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C92" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D92" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E92" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F92" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G92" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C93" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D93" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E93" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F93" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G93" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C94" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E94" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F94" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G94" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B95" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C95" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D95" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E95" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F95" s="8" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G95" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B96" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C96" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D96" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F96" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G96" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B97" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C97" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D97" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E97" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F97" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G97" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B98" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C98" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E98" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F98" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G98" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B99" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C99" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D99" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E99" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F99" s="8" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G99" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B100" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C100" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D100" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E100" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F100" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G100" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B101" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C101" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D101" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E101" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F101" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G101" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B102" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E102" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F102" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G102" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E103" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F103" s="8" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G103" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C104" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D104" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E104" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F104" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G104" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B105" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C105" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D105" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E105" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F105" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G105" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C106" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E106" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F106" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G106" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C107" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D107" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E107" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F107" s="8" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G107" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C108" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D108" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E108" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F108" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G108" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C109" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D109" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E109" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F109" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G109" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10429,7 +12398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -12850,6 +14819,546 @@
         <v>7.75</v>
       </c>
       <c r="G89" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B90" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C90" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E90" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F90" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G90" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B91" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C91" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E91" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F91" s="8" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="G91" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B92" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C92" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D92" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E92" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F92" s="8" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G92" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C93" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D93" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E93" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F93" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G93" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C94" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E94" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F94" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G94" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B95" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C95" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D95" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E95" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F95" s="8" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="G95" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B96" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C96" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D96" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F96" s="8" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G96" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B97" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C97" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D97" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E97" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F97" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G97" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B98" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C98" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E98" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F98" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G98" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B99" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C99" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D99" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E99" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F99" s="8" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="G99" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B100" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C100" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D100" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E100" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F100" s="8" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G100" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B101" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C101" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D101" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E101" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F101" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G101" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B102" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E102" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F102" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G102" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E103" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F103" s="8" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="G103" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C104" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D104" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E104" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F104" s="8" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G104" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B105" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C105" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D105" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E105" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F105" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G105" s="9" t="n">
+        <v>46167.54166666666</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C106" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E106" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F106" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G106" s="9" t="n">
+        <v>46078.54166666666</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C107" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D107" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E107" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F107" s="8" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="G107" s="9" t="n">
+        <v>46106.54166666666</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C108" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D108" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E108" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F108" s="8" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G108" s="9" t="n">
+        <v>46137.54166666666</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>marcos</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAM VERM POLO </t>
+        </is>
+      </c>
+      <c r="C109" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D109" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="E109" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="F109" s="8" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G109" s="9" t="n">
         <v>46167.54166666666</v>
       </c>
     </row>

</xml_diff>